<commit_message>
update Painless solver option
</commit_message>
<xml_diff>
--- a/result/verified/j30_Bimerge_BDD.xlsx
+++ b/result/verified/j30_Bimerge_BDD.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">MRCPSP_j30_results_20250909_005!$A$1:$I$641</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr/>
@@ -2478,9 +2478,15 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2802,10 +2808,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I641"/>
+  <dimension ref="A1:M641"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2833,8 +2839,16 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K1">
+        <f>COUNTIF(F:F, "Optimal")</f>
+        <v>545</v>
+      </c>
+      <c r="M1">
+        <f>AVERAGE(G2:G641)</f>
+        <v>82.775703124999964</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2860,7 +2874,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -2886,7 +2900,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -2912,7 +2926,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -2938,7 +2952,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -2964,7 +2978,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -2990,7 +3004,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -3016,7 +3030,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -3042,7 +3056,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -3068,7 +3082,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -3094,7 +3108,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -3120,7 +3134,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -3146,7 +3160,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -3172,7 +3186,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>24</v>
       </c>
@@ -3198,7 +3212,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -12686,16 +12700,16 @@
         <v>1484536</v>
       </c>
       <c r="E385">
-        <v>44</v>
-      </c>
-      <c r="F385" t="s">
-        <v>43</v>
-      </c>
-      <c r="G385">
-        <v>3601.22</v>
+        <v>42</v>
+      </c>
+      <c r="F385" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G385" s="3">
+        <v>2461.48</v>
       </c>
       <c r="H385" t="s">
-        <v>44</v>
+        <v>11</v>
       </c>
     </row>
     <row r="386" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>